<commit_message>
Use Russian label for publication address
</commit_message>
<xml_diff>
--- a/docs/sample-blog-platform.xlsx
+++ b/docs/sample-blog-platform.xlsx
@@ -64,7 +64,7 @@
     <t>Заголовок</t>
   </si>
   <si>
-    <t>Slug</t>
+    <t>Адрес публикации</t>
   </si>
   <si>
     <t>Статус</t>
@@ -381,10 +381,10 @@
         <v>22</v>
       </c>
       <c r="F2" t="n" s="2">
-        <v>46263.64716702546</v>
+        <v>46269.675964270835</v>
       </c>
       <c r="G2" t="n" s="2">
-        <v>46264.64716702546</v>
+        <v>46270.675964270835</v>
       </c>
       <c r="H2" t="s" s="0">
         <v>23</v>
@@ -407,10 +407,10 @@
         <v>22</v>
       </c>
       <c r="F3" t="n" s="2">
-        <v>46265.64716702546</v>
+        <v>46271.675964270835</v>
       </c>
       <c r="G3" t="n" s="2">
-        <v>46266.64716702546</v>
+        <v>46272.675964270835</v>
       </c>
       <c r="H3" t="s" s="0">
         <v>26</v>
@@ -433,7 +433,7 @@
         <v>29</v>
       </c>
       <c r="F4" t="n" s="2">
-        <v>46268.64716702546</v>
+        <v>46274.675964270835</v>
       </c>
       <c r="G4" s="0"/>
       <c r="H4" t="s" s="0">
@@ -457,7 +457,7 @@
         <v>33</v>
       </c>
       <c r="F5" t="n" s="2">
-        <v>46271.64716702546</v>
+        <v>46277.675964270835</v>
       </c>
       <c r="G5" s="0"/>
       <c r="H5" t="s" s="0">
@@ -481,10 +481,10 @@
         <v>22</v>
       </c>
       <c r="F6" t="n" s="2">
-        <v>46273.64716702546</v>
+        <v>46279.675964270835</v>
       </c>
       <c r="G6" t="n" s="2">
-        <v>46274.64716702546</v>
+        <v>46280.675964270835</v>
       </c>
       <c r="H6" t="s" s="0">
         <v>37</v>
@@ -507,7 +507,7 @@
         <v>29</v>
       </c>
       <c r="F7" t="n" s="2">
-        <v>46275.64716702546</v>
+        <v>46281.675964270835</v>
       </c>
       <c r="G7" s="0"/>
       <c r="H7" t="s" s="0">
@@ -531,7 +531,7 @@
         <v>33</v>
       </c>
       <c r="F8" t="n" s="2">
-        <v>46276.64716702546</v>
+        <v>46282.675964270835</v>
       </c>
       <c r="G8" s="0"/>
       <c r="H8" t="s" s="0">
@@ -555,10 +555,10 @@
         <v>22</v>
       </c>
       <c r="F9" t="n" s="2">
-        <v>46277.64716702546</v>
+        <v>46283.675964270835</v>
       </c>
       <c r="G9" t="n" s="2">
-        <v>46278.64716702546</v>
+        <v>46284.675964270835</v>
       </c>
       <c r="H9" t="s" s="0">
         <v>46</v>
@@ -581,10 +581,10 @@
         <v>49</v>
       </c>
       <c r="F10" t="n" s="2">
-        <v>46253.64716702546</v>
+        <v>46259.675964270835</v>
       </c>
       <c r="G10" t="n" s="2">
-        <v>46254.64716702546</v>
+        <v>46260.675964270835</v>
       </c>
       <c r="H10" t="s" s="0">
         <v>50</v>
@@ -607,7 +607,7 @@
         <v>33</v>
       </c>
       <c r="F11" t="n" s="2">
-        <v>46281.64716702546</v>
+        <v>46287.675964270835</v>
       </c>
       <c r="G11" s="0"/>
       <c r="H11" t="s" s="0">

</xml_diff>

<commit_message>
Translate publication statuses for users
</commit_message>
<xml_diff>
--- a/docs/sample-blog-platform.xlsx
+++ b/docs/sample-blog-platform.xlsx
@@ -85,7 +85,7 @@
     <t>blog-platform-architecture</t>
   </si>
   <si>
-    <t>PUBLISHED</t>
+    <t>Опубликована</t>
   </si>
   <si>
     <t>Обзор основных слоев приложения и их ответственности.</t>
@@ -106,7 +106,7 @@
     <t>java-collections</t>
   </si>
   <si>
-    <t>REVIEW</t>
+    <t>На проверке</t>
   </si>
   <si>
     <t>Фильтрация и сортировка публикаций с использованием Stream API.</t>
@@ -118,7 +118,7 @@
     <t>postgresql-draft</t>
   </si>
   <si>
-    <t>DRAFT</t>
+    <t>Черновик</t>
   </si>
   <si>
     <t>Заметки о проектировании таблиц и ограничений.</t>
@@ -166,7 +166,7 @@
     <t>first-platform-version</t>
   </si>
   <si>
-    <t>ARCHIVED</t>
+    <t>В архиве</t>
   </si>
   <si>
     <t>Архивная публикация о первой версии проекта.</t>
@@ -332,7 +332,7 @@
     <col min="2" max="2" width="10.91015625" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="28.37109375" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="23.88671875" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="11.1328125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="14.25390625" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="16.90234375" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="16.90234375" customWidth="true" bestFit="true"/>
     <col min="8" max="8" width="60.0" customWidth="true" bestFit="true"/>

</xml_diff>